<commit_message>
2.1-2.5 revised and updated
</commit_message>
<xml_diff>
--- a/project_plan.xlsx
+++ b/project_plan.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06DDE32-3A60-4566-B1A1-F5D1EA0633F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13170" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="4" r:id="rId1"/>
@@ -17,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sprint Backlog'!$A$2:$J$181</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,13 +34,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Author</author>
-    <author>tc={148E080D-CE22-4CE0-8311-B67C30FEF121}</author>
   </authors>
   <commentList>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="E5" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -58,12 +56,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="E6" authorId="1" shapeId="0" xr:uid="{148E080D-CE22-4CE0-8311-B67C30FEF121}">
+    <comment ref="E6" authorId="0" shapeId="0">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Get client verification</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -71,12 +78,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="H2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -102,7 +109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="C3" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -126,7 +133,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+    <comment ref="C12" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -150,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
+    <comment ref="C15" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -174,7 +181,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
+    <comment ref="C18" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -198,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
+    <comment ref="C26" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -223,7 +230,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
+    <comment ref="C29" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -247,7 +254,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008000000}">
+    <comment ref="C31" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -271,7 +278,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009000000}">
+    <comment ref="C38" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -295,7 +302,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000A000000}">
+    <comment ref="C46" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -319,7 +326,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B000000}">
+    <comment ref="C50" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -343,7 +350,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000C000000}">
+    <comment ref="C59" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -367,7 +374,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C65" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D000000}">
+    <comment ref="C65" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -391,7 +398,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C77" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E000000}">
+    <comment ref="C77" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -415,7 +422,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C88" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F000000}">
+    <comment ref="C88" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -439,7 +446,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C101" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000010000000}">
+    <comment ref="C101" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -463,7 +470,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C110" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000011000000}">
+    <comment ref="C110" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -487,7 +494,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C116" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000012000000}">
+    <comment ref="C116" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -511,7 +518,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C127" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000013000000}">
+    <comment ref="C127" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -535,7 +542,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C137" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000014000000}">
+    <comment ref="C137" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -559,7 +566,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C142" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000015000000}">
+    <comment ref="C142" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -583,7 +590,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C157" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000016000000}">
+    <comment ref="C157" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -607,7 +614,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C161" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000017000000}">
+    <comment ref="C161" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -631,7 +638,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C168" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000018000000}">
+    <comment ref="C168" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -655,7 +662,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C174" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000019000000}">
+    <comment ref="C174" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -684,12 +691,12 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="H2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -720,14 +727,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -2593,7 +2600,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="11">
     <font>
       <sz val="11"/>
@@ -2889,16 +2896,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2908,17 +2918,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4105,9 +4112,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4145,9 +4152,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4182,7 +4189,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4217,7 +4224,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4398,25 +4405,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" customWidth="1"/>
-    <col min="5" max="5" width="51.109375" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" customWidth="1"/>
+    <col min="5" max="5" width="51.140625" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="10"/>
-      <c r="B1" s="47" t="s">
+      <c r="B1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10"/>
     </row>
@@ -4440,7 +4447,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="100.8">
+    <row r="3" spans="1:6" ht="105">
       <c r="A3" s="16">
         <v>1</v>
       </c>
@@ -4491,7 +4498,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="86.4">
+    <row r="6" spans="1:6" ht="90">
       <c r="A6" s="15">
         <v>4</v>
       </c>
@@ -4542,32 +4549,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J181"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="74.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
     </row>
     <row r="2" spans="1:10" s="4" customFormat="1">
       <c r="A2" s="10" t="s">
@@ -4602,632 +4609,632 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="50">
+      <c r="A3" s="51">
         <v>1</v>
       </c>
-      <c r="B3" s="51">
+      <c r="B3" s="45">
         <v>1</v>
       </c>
-      <c r="C3" s="51">
+      <c r="C3" s="45">
         <v>1.1000000000000001</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="48" cm="1">
+      <c r="F3" s="49" cm="1">
         <f t="array" ref="F3">_xlfn.SWITCH(E3,"XS",1,"S",2,"M",3,"L",5,"XL",8,"XXL",13,"XXXL",21,"")</f>
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="50"/>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
+      <c r="A4" s="51"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
       <c r="D4" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="50"/>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
+      <c r="A5" s="51"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="50"/>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
+      <c r="A6" s="51"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="50"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
+      <c r="A7" s="51"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
       <c r="D7" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="50"/>
-      <c r="B8" s="51"/>
-      <c r="C8" s="51"/>
+      <c r="A8" s="51"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
       <c r="D8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="50"/>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
+      <c r="A9" s="51"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="50"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
       <c r="D10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="50"/>
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
+      <c r="A11" s="51"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
       <c r="D11" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="48"/>
-      <c r="F11" s="48"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="50"/>
-      <c r="B12" s="51"/>
-      <c r="C12" s="51">
+      <c r="A12" s="51"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45">
         <v>1.2</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="48" t="s">
+      <c r="E12" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="48" cm="1">
+      <c r="F12" s="49" cm="1">
         <f t="array" ref="F12">_xlfn.SWITCH(E3,"XS",1,"S",2,"M",3,"L",5,"XL",8,"XXL",13,"XXXL",21,"")</f>
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="50"/>
-      <c r="B13" s="51"/>
-      <c r="C13" s="51"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
       <c r="D13" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="50"/>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="45"/>
       <c r="D14" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="50"/>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51">
+      <c r="A15" s="51"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45">
         <v>1.3</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="48"/>
+      <c r="F15" s="49"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="50"/>
-      <c r="B16" s="51"/>
-      <c r="C16" s="51"/>
+      <c r="A16" s="51"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
       <c r="D16" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="50"/>
-      <c r="B17" s="51"/>
-      <c r="C17" s="51"/>
+      <c r="A17" s="51"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
       <c r="D17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="50"/>
-      <c r="B18" s="51"/>
-      <c r="C18" s="51">
+      <c r="A18" s="51"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45">
         <v>1.4</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="48" t="s">
+      <c r="E18" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="48"/>
+      <c r="F18" s="49"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="50"/>
-      <c r="B19" s="51"/>
-      <c r="C19" s="51"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
       <c r="D19" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="50"/>
-      <c r="B20" s="51"/>
-      <c r="C20" s="51"/>
+      <c r="A20" s="51"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
       <c r="D20" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="50"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="51"/>
+      <c r="A21" s="51"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
       <c r="D21" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="50"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="51"/>
+      <c r="A22" s="51"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
       <c r="D22" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="50"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="51"/>
+      <c r="A23" s="51"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
       <c r="D23" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="50"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
+      <c r="A24" s="51"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
       <c r="D24" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="50"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="45"/>
       <c r="D25" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="50"/>
+      <c r="A26" s="51"/>
       <c r="B26" s="52">
         <v>2</v>
       </c>
-      <c r="C26" s="51">
+      <c r="C26" s="45">
         <v>2.1</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E26" s="49" t="s">
+      <c r="E26" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="48"/>
+      <c r="F26" s="49"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="50"/>
+      <c r="A27" s="51"/>
       <c r="B27" s="52"/>
-      <c r="C27" s="51"/>
+      <c r="C27" s="45"/>
       <c r="D27" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="49"/>
-      <c r="F27" s="48"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="49"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="50"/>
+      <c r="A28" s="51"/>
       <c r="B28" s="52"/>
-      <c r="C28" s="51"/>
+      <c r="C28" s="45"/>
       <c r="D28" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="E28" s="49"/>
-      <c r="F28" s="48"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="49"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="50"/>
+      <c r="A29" s="51"/>
       <c r="B29" s="52"/>
-      <c r="C29" s="53">
+      <c r="C29" s="47">
         <v>2.2000000000000002</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="48" t="s">
+      <c r="E29" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="48"/>
+      <c r="F29" s="49"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="50"/>
+      <c r="A30" s="51"/>
       <c r="B30" s="52"/>
-      <c r="C30" s="53"/>
+      <c r="C30" s="47"/>
       <c r="D30" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="50"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="52"/>
-      <c r="C31" s="51">
+      <c r="C31" s="45">
         <v>2.2999999999999998</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E31" s="48" t="s">
+      <c r="E31" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48" t="s">
+      <c r="F31" s="49"/>
+      <c r="G31" s="49" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="50"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="52"/>
-      <c r="C32" s="51"/>
+      <c r="C32" s="45"/>
       <c r="D32" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="48"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="48"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="50"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="52"/>
-      <c r="C33" s="51"/>
+      <c r="C33" s="45"/>
       <c r="D33" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="50"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="52"/>
-      <c r="C34" s="51"/>
+      <c r="C34" s="45"/>
       <c r="D34" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="48"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="49"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="50"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="52"/>
-      <c r="C35" s="51"/>
+      <c r="C35" s="45"/>
       <c r="D35" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="50"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="52"/>
-      <c r="C36" s="51"/>
+      <c r="C36" s="45"/>
       <c r="D36" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="50"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="52"/>
-      <c r="C37" s="51"/>
+      <c r="C37" s="45"/>
       <c r="D37" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="49"/>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="50"/>
+      <c r="A38" s="51"/>
       <c r="B38" s="52"/>
-      <c r="C38" s="51">
+      <c r="C38" s="45">
         <v>2.4</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="48" t="s">
+      <c r="E38" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="48"/>
+      <c r="F38" s="49"/>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="50"/>
+      <c r="A39" s="51"/>
       <c r="B39" s="52"/>
-      <c r="C39" s="51"/>
+      <c r="C39" s="45"/>
       <c r="D39" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="50"/>
+      <c r="A40" s="51"/>
       <c r="B40" s="52"/>
-      <c r="C40" s="51"/>
+      <c r="C40" s="45"/>
       <c r="D40" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="50"/>
+      <c r="A41" s="51"/>
       <c r="B41" s="52"/>
-      <c r="C41" s="51"/>
+      <c r="C41" s="45"/>
       <c r="D41" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="50"/>
+      <c r="A42" s="51"/>
       <c r="B42" s="52"/>
-      <c r="C42" s="51"/>
+      <c r="C42" s="45"/>
       <c r="D42" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="50"/>
+      <c r="A43" s="51"/>
       <c r="B43" s="52"/>
-      <c r="C43" s="51"/>
+      <c r="C43" s="45"/>
       <c r="D43" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="48"/>
-      <c r="F43" s="48"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="50"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="52"/>
-      <c r="C44" s="51"/>
+      <c r="C44" s="45"/>
       <c r="D44" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="E44" s="48"/>
-      <c r="F44" s="48"/>
+      <c r="E44" s="49"/>
+      <c r="F44" s="49"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="50"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="52"/>
-      <c r="C45" s="51"/>
+      <c r="C45" s="45"/>
       <c r="D45" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="50"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="52"/>
-      <c r="C46" s="51">
+      <c r="C46" s="45">
         <v>2.5</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E46" s="49" t="s">
+      <c r="E46" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="F46" s="48"/>
+      <c r="F46" s="49"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="50"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="52"/>
-      <c r="C47" s="51"/>
+      <c r="C47" s="45"/>
       <c r="D47" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E47" s="49"/>
-      <c r="F47" s="48"/>
+      <c r="E47" s="50"/>
+      <c r="F47" s="49"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="50"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="52"/>
-      <c r="C48" s="51"/>
+      <c r="C48" s="45"/>
       <c r="D48" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E48" s="49"/>
-      <c r="F48" s="48"/>
+      <c r="E48" s="50"/>
+      <c r="F48" s="49"/>
     </row>
     <row r="49" spans="1:6">
-      <c r="A49" s="50"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="52"/>
-      <c r="C49" s="51"/>
+      <c r="C49" s="45"/>
       <c r="D49" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E49" s="49"/>
-      <c r="F49" s="48"/>
+      <c r="E49" s="50"/>
+      <c r="F49" s="49"/>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="50"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="52"/>
-      <c r="C50" s="51">
+      <c r="C50" s="45">
         <v>2.7</v>
       </c>
       <c r="D50" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E50" s="48" t="s">
+      <c r="E50" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F50" s="48"/>
+      <c r="F50" s="49"/>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="50"/>
+      <c r="A51" s="51"/>
       <c r="B51" s="52"/>
-      <c r="C51" s="51"/>
+      <c r="C51" s="45"/>
       <c r="D51" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E51" s="48"/>
-      <c r="F51" s="48"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="50"/>
+      <c r="A52" s="51"/>
       <c r="B52" s="52"/>
-      <c r="C52" s="51"/>
+      <c r="C52" s="45"/>
       <c r="D52" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E52" s="48"/>
-      <c r="F52" s="48"/>
+      <c r="E52" s="49"/>
+      <c r="F52" s="49"/>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="50"/>
+      <c r="A53" s="51"/>
       <c r="B53" s="52"/>
-      <c r="C53" s="51"/>
+      <c r="C53" s="45"/>
       <c r="D53" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E53" s="48"/>
-      <c r="F53" s="48"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
     </row>
     <row r="54" spans="1:6">
-      <c r="A54" s="50"/>
+      <c r="A54" s="51"/>
       <c r="B54" s="52"/>
-      <c r="C54" s="51"/>
+      <c r="C54" s="45"/>
       <c r="D54" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E54" s="48"/>
-      <c r="F54" s="48"/>
+      <c r="E54" s="49"/>
+      <c r="F54" s="49"/>
     </row>
     <row r="55" spans="1:6">
-      <c r="A55" s="50"/>
+      <c r="A55" s="51"/>
       <c r="B55" s="52"/>
-      <c r="C55" s="51"/>
+      <c r="C55" s="45"/>
       <c r="D55" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E55" s="48"/>
-      <c r="F55" s="48"/>
+      <c r="E55" s="49"/>
+      <c r="F55" s="49"/>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="50"/>
+      <c r="A56" s="51"/>
       <c r="B56" s="52"/>
-      <c r="C56" s="51"/>
+      <c r="C56" s="45"/>
       <c r="D56" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E56" s="48"/>
-      <c r="F56" s="48"/>
+      <c r="E56" s="49"/>
+      <c r="F56" s="49"/>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="50"/>
+      <c r="A57" s="51"/>
       <c r="B57" s="52"/>
-      <c r="C57" s="51"/>
+      <c r="C57" s="45"/>
       <c r="D57" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E57" s="48"/>
-      <c r="F57" s="48"/>
+      <c r="E57" s="49"/>
+      <c r="F57" s="49"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="50"/>
+      <c r="A58" s="51"/>
       <c r="B58" s="52"/>
-      <c r="C58" s="51"/>
+      <c r="C58" s="45"/>
       <c r="D58" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E58" s="48"/>
-      <c r="F58" s="48"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="20"/>
-      <c r="B59" s="51">
+      <c r="B59" s="45">
         <v>3</v>
       </c>
-      <c r="C59" s="51">
+      <c r="C59" s="45">
         <v>3.1</v>
       </c>
       <c r="D59" s="7" t="s">
@@ -5236,48 +5243,48 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="19"/>
-      <c r="B60" s="51"/>
-      <c r="C60" s="51"/>
+      <c r="B60" s="45"/>
+      <c r="C60" s="45"/>
       <c r="D60" s="7" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="19"/>
-      <c r="B61" s="51"/>
-      <c r="C61" s="51"/>
+      <c r="B61" s="45"/>
+      <c r="C61" s="45"/>
       <c r="D61" s="7" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="19"/>
-      <c r="B62" s="51"/>
-      <c r="C62" s="51"/>
+      <c r="B62" s="45"/>
+      <c r="C62" s="45"/>
       <c r="D62" s="7" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="19"/>
-      <c r="B63" s="51"/>
-      <c r="C63" s="51"/>
+      <c r="B63" s="45"/>
+      <c r="C63" s="45"/>
       <c r="D63" s="7" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="19"/>
-      <c r="B64" s="51"/>
-      <c r="C64" s="51"/>
+      <c r="B64" s="45"/>
+      <c r="C64" s="45"/>
       <c r="D64" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="19"/>
-      <c r="B65" s="51"/>
-      <c r="C65" s="51">
+      <c r="B65" s="45"/>
+      <c r="C65" s="45">
         <v>3.2</v>
       </c>
       <c r="D65" s="7" t="s">
@@ -5286,96 +5293,96 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="19"/>
-      <c r="B66" s="51"/>
-      <c r="C66" s="51"/>
+      <c r="B66" s="45"/>
+      <c r="C66" s="45"/>
       <c r="D66" s="7" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="19"/>
-      <c r="B67" s="51"/>
-      <c r="C67" s="51"/>
+      <c r="B67" s="45"/>
+      <c r="C67" s="45"/>
       <c r="D67" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="19"/>
-      <c r="B68" s="51"/>
-      <c r="C68" s="51"/>
+      <c r="B68" s="45"/>
+      <c r="C68" s="45"/>
       <c r="D68" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="19"/>
-      <c r="B69" s="51"/>
-      <c r="C69" s="51"/>
+      <c r="B69" s="45"/>
+      <c r="C69" s="45"/>
       <c r="D69" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="19"/>
-      <c r="B70" s="51"/>
-      <c r="C70" s="51"/>
+      <c r="B70" s="45"/>
+      <c r="C70" s="45"/>
       <c r="D70" s="7" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="19"/>
-      <c r="B71" s="51"/>
-      <c r="C71" s="51"/>
+      <c r="B71" s="45"/>
+      <c r="C71" s="45"/>
       <c r="D71" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="19"/>
-      <c r="B72" s="51"/>
-      <c r="C72" s="51"/>
+      <c r="B72" s="45"/>
+      <c r="C72" s="45"/>
       <c r="D72" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="19"/>
-      <c r="B73" s="51"/>
-      <c r="C73" s="51"/>
+      <c r="B73" s="45"/>
+      <c r="C73" s="45"/>
       <c r="D73" s="7" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="19"/>
-      <c r="B74" s="51"/>
-      <c r="C74" s="51"/>
+      <c r="B74" s="45"/>
+      <c r="C74" s="45"/>
       <c r="D74" s="7" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="19"/>
-      <c r="B75" s="51"/>
-      <c r="C75" s="51"/>
+      <c r="B75" s="45"/>
+      <c r="C75" s="45"/>
       <c r="D75" s="7" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="19"/>
-      <c r="B76" s="51"/>
-      <c r="C76" s="51"/>
+      <c r="B76" s="45"/>
+      <c r="C76" s="45"/>
       <c r="D76" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="19"/>
-      <c r="B77" s="51"/>
-      <c r="C77" s="51">
+      <c r="B77" s="45"/>
+      <c r="C77" s="45">
         <v>3.3</v>
       </c>
       <c r="D77" s="7" t="s">
@@ -5384,88 +5391,88 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="19"/>
-      <c r="B78" s="51"/>
-      <c r="C78" s="51"/>
+      <c r="B78" s="45"/>
+      <c r="C78" s="45"/>
       <c r="D78" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="19"/>
-      <c r="B79" s="51"/>
-      <c r="C79" s="51"/>
+      <c r="B79" s="45"/>
+      <c r="C79" s="45"/>
       <c r="D79" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="19"/>
-      <c r="B80" s="51"/>
-      <c r="C80" s="51"/>
+      <c r="B80" s="45"/>
+      <c r="C80" s="45"/>
       <c r="D80" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="19"/>
-      <c r="B81" s="51"/>
-      <c r="C81" s="51"/>
+      <c r="B81" s="45"/>
+      <c r="C81" s="45"/>
       <c r="D81" s="7" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="19"/>
-      <c r="B82" s="51"/>
-      <c r="C82" s="51"/>
+      <c r="B82" s="45"/>
+      <c r="C82" s="45"/>
       <c r="D82" s="7" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="19"/>
-      <c r="B83" s="51"/>
-      <c r="C83" s="51"/>
+      <c r="B83" s="45"/>
+      <c r="C83" s="45"/>
       <c r="D83" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="19"/>
-      <c r="B84" s="51"/>
-      <c r="C84" s="51"/>
+      <c r="B84" s="45"/>
+      <c r="C84" s="45"/>
       <c r="D84" s="7" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="19"/>
-      <c r="B85" s="51"/>
-      <c r="C85" s="51"/>
+      <c r="B85" s="45"/>
+      <c r="C85" s="45"/>
       <c r="D85" s="7" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="19"/>
-      <c r="B86" s="51"/>
-      <c r="C86" s="51"/>
+      <c r="B86" s="45"/>
+      <c r="C86" s="45"/>
       <c r="D86" s="7" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="19"/>
-      <c r="B87" s="51"/>
-      <c r="C87" s="51"/>
+      <c r="B87" s="45"/>
+      <c r="C87" s="45"/>
       <c r="D87" s="7" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="19"/>
-      <c r="B88" s="51"/>
-      <c r="C88" s="51">
+      <c r="B88" s="45"/>
+      <c r="C88" s="45">
         <v>3.4</v>
       </c>
       <c r="D88" s="15" t="s">
@@ -5474,104 +5481,104 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="19"/>
-      <c r="B89" s="51"/>
-      <c r="C89" s="51"/>
+      <c r="B89" s="45"/>
+      <c r="C89" s="45"/>
       <c r="D89" s="7" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="19"/>
-      <c r="B90" s="51"/>
-      <c r="C90" s="51"/>
+      <c r="B90" s="45"/>
+      <c r="C90" s="45"/>
       <c r="D90" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="19"/>
-      <c r="B91" s="51"/>
-      <c r="C91" s="51"/>
+      <c r="B91" s="45"/>
+      <c r="C91" s="45"/>
       <c r="D91" s="7" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="19"/>
-      <c r="B92" s="51"/>
-      <c r="C92" s="51"/>
+      <c r="B92" s="45"/>
+      <c r="C92" s="45"/>
       <c r="D92" s="7" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="19"/>
-      <c r="B93" s="51"/>
-      <c r="C93" s="51"/>
+      <c r="B93" s="45"/>
+      <c r="C93" s="45"/>
       <c r="D93" s="7" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="19"/>
-      <c r="B94" s="51"/>
-      <c r="C94" s="51"/>
+      <c r="B94" s="45"/>
+      <c r="C94" s="45"/>
       <c r="D94" s="7" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="19"/>
-      <c r="B95" s="51"/>
-      <c r="C95" s="51"/>
+      <c r="B95" s="45"/>
+      <c r="C95" s="45"/>
       <c r="D95" s="7" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="19"/>
-      <c r="B96" s="51"/>
-      <c r="C96" s="51"/>
+      <c r="B96" s="45"/>
+      <c r="C96" s="45"/>
       <c r="D96" s="7" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="19"/>
-      <c r="B97" s="51"/>
-      <c r="C97" s="51"/>
+      <c r="B97" s="45"/>
+      <c r="C97" s="45"/>
       <c r="D97" s="7" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="19"/>
-      <c r="B98" s="51"/>
-      <c r="C98" s="51"/>
+      <c r="B98" s="45"/>
+      <c r="C98" s="45"/>
       <c r="D98" s="7" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="19"/>
-      <c r="B99" s="51"/>
-      <c r="C99" s="51"/>
+      <c r="B99" s="45"/>
+      <c r="C99" s="45"/>
       <c r="D99" s="7" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="19"/>
-      <c r="B100" s="51"/>
-      <c r="C100" s="51"/>
+      <c r="B100" s="45"/>
+      <c r="C100" s="45"/>
       <c r="D100" s="7" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="19"/>
-      <c r="B101" s="51"/>
-      <c r="C101" s="51">
+      <c r="B101" s="45"/>
+      <c r="C101" s="45">
         <v>3.5</v>
       </c>
       <c r="D101" s="11" t="s">
@@ -5580,72 +5587,72 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="19"/>
-      <c r="B102" s="51"/>
-      <c r="C102" s="51"/>
+      <c r="B102" s="45"/>
+      <c r="C102" s="45"/>
       <c r="D102" s="7" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="19"/>
-      <c r="B103" s="51"/>
-      <c r="C103" s="51"/>
+      <c r="B103" s="45"/>
+      <c r="C103" s="45"/>
       <c r="D103" s="7" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="19"/>
-      <c r="B104" s="51"/>
-      <c r="C104" s="51"/>
+      <c r="B104" s="45"/>
+      <c r="C104" s="45"/>
       <c r="D104" s="7" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="19"/>
-      <c r="B105" s="51"/>
-      <c r="C105" s="51"/>
+      <c r="B105" s="45"/>
+      <c r="C105" s="45"/>
       <c r="D105" s="7" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="19"/>
-      <c r="B106" s="51"/>
-      <c r="C106" s="51"/>
+      <c r="B106" s="45"/>
+      <c r="C106" s="45"/>
       <c r="D106" s="7" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="19"/>
-      <c r="B107" s="51"/>
-      <c r="C107" s="51"/>
+      <c r="B107" s="45"/>
+      <c r="C107" s="45"/>
       <c r="D107" s="7" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="19"/>
-      <c r="B108" s="51"/>
-      <c r="C108" s="51"/>
+      <c r="B108" s="45"/>
+      <c r="C108" s="45"/>
       <c r="D108" s="7" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="19"/>
-      <c r="B109" s="51"/>
-      <c r="C109" s="51"/>
+      <c r="B109" s="45"/>
+      <c r="C109" s="45"/>
       <c r="D109" s="7" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="19"/>
-      <c r="B110" s="51"/>
-      <c r="C110" s="51">
+      <c r="B110" s="45"/>
+      <c r="C110" s="45">
         <v>3.6</v>
       </c>
       <c r="D110" s="7" t="s">
@@ -5654,48 +5661,48 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="19"/>
-      <c r="B111" s="51"/>
-      <c r="C111" s="51"/>
+      <c r="B111" s="45"/>
+      <c r="C111" s="45"/>
       <c r="D111" s="7" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="19"/>
-      <c r="B112" s="51"/>
-      <c r="C112" s="51"/>
+      <c r="B112" s="45"/>
+      <c r="C112" s="45"/>
       <c r="D112" s="7" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="19"/>
-      <c r="B113" s="51"/>
-      <c r="C113" s="51"/>
+      <c r="B113" s="45"/>
+      <c r="C113" s="45"/>
       <c r="D113" s="7" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="19"/>
-      <c r="B114" s="51"/>
-      <c r="C114" s="51"/>
+      <c r="B114" s="45"/>
+      <c r="C114" s="45"/>
       <c r="D114" s="7" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="19"/>
-      <c r="B115" s="51"/>
-      <c r="C115" s="51"/>
+      <c r="B115" s="45"/>
+      <c r="C115" s="45"/>
       <c r="D115" s="7" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="19"/>
-      <c r="B116" s="51"/>
-      <c r="C116" s="51">
+      <c r="B116" s="45"/>
+      <c r="C116" s="45">
         <v>3.7</v>
       </c>
       <c r="D116" s="7" t="s">
@@ -5704,88 +5711,88 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="19"/>
-      <c r="B117" s="51"/>
-      <c r="C117" s="51"/>
+      <c r="B117" s="45"/>
+      <c r="C117" s="45"/>
       <c r="D117" s="7" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="19"/>
-      <c r="B118" s="51"/>
-      <c r="C118" s="51"/>
+      <c r="B118" s="45"/>
+      <c r="C118" s="45"/>
       <c r="D118" s="7" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="19"/>
-      <c r="B119" s="51"/>
-      <c r="C119" s="51"/>
+      <c r="B119" s="45"/>
+      <c r="C119" s="45"/>
       <c r="D119" s="7" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="19"/>
-      <c r="B120" s="51"/>
-      <c r="C120" s="51"/>
+      <c r="B120" s="45"/>
+      <c r="C120" s="45"/>
       <c r="D120" s="7" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="19"/>
-      <c r="B121" s="51"/>
-      <c r="C121" s="51"/>
+      <c r="B121" s="45"/>
+      <c r="C121" s="45"/>
       <c r="D121" s="7" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="19"/>
-      <c r="B122" s="51"/>
-      <c r="C122" s="51"/>
+      <c r="B122" s="45"/>
+      <c r="C122" s="45"/>
       <c r="D122" s="7" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="19"/>
-      <c r="B123" s="51"/>
-      <c r="C123" s="51"/>
+      <c r="B123" s="45"/>
+      <c r="C123" s="45"/>
       <c r="D123" s="7" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="19"/>
-      <c r="B124" s="51"/>
-      <c r="C124" s="51"/>
+      <c r="B124" s="45"/>
+      <c r="C124" s="45"/>
       <c r="D124" s="7" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="19"/>
-      <c r="B125" s="51"/>
-      <c r="C125" s="51"/>
+      <c r="B125" s="45"/>
+      <c r="C125" s="45"/>
       <c r="D125" s="7" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="19"/>
-      <c r="B126" s="51"/>
-      <c r="C126" s="51"/>
+      <c r="B126" s="45"/>
+      <c r="C126" s="45"/>
       <c r="D126" s="7" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="19"/>
-      <c r="B127" s="51"/>
-      <c r="C127" s="51">
+      <c r="B127" s="45"/>
+      <c r="C127" s="45">
         <v>3.8</v>
       </c>
       <c r="D127" s="7" t="s">
@@ -5794,80 +5801,80 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="19"/>
-      <c r="B128" s="51"/>
-      <c r="C128" s="51"/>
+      <c r="B128" s="45"/>
+      <c r="C128" s="45"/>
       <c r="D128" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="19"/>
-      <c r="B129" s="51"/>
-      <c r="C129" s="51"/>
+      <c r="B129" s="45"/>
+      <c r="C129" s="45"/>
       <c r="D129" s="7" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="19"/>
-      <c r="B130" s="51"/>
-      <c r="C130" s="51"/>
+      <c r="B130" s="45"/>
+      <c r="C130" s="45"/>
       <c r="D130" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="19"/>
-      <c r="B131" s="51"/>
-      <c r="C131" s="51"/>
+      <c r="B131" s="45"/>
+      <c r="C131" s="45"/>
       <c r="D131" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="19"/>
-      <c r="B132" s="51"/>
-      <c r="C132" s="51"/>
+      <c r="B132" s="45"/>
+      <c r="C132" s="45"/>
       <c r="D132" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="19"/>
-      <c r="B133" s="51"/>
-      <c r="C133" s="51"/>
+      <c r="B133" s="45"/>
+      <c r="C133" s="45"/>
       <c r="D133" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="19"/>
-      <c r="B134" s="51"/>
-      <c r="C134" s="51"/>
+      <c r="B134" s="45"/>
+      <c r="C134" s="45"/>
       <c r="D134" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="19"/>
-      <c r="B135" s="51"/>
-      <c r="C135" s="51"/>
+      <c r="B135" s="45"/>
+      <c r="C135" s="45"/>
       <c r="D135" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="19"/>
-      <c r="B136" s="51"/>
-      <c r="C136" s="51"/>
+      <c r="B136" s="45"/>
+      <c r="C136" s="45"/>
       <c r="D136" s="7" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="19"/>
-      <c r="B137" s="51"/>
-      <c r="C137" s="51">
+      <c r="B137" s="45"/>
+      <c r="C137" s="45">
         <v>3.9</v>
       </c>
       <c r="D137" s="7" t="s">
@@ -5876,40 +5883,40 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="19"/>
-      <c r="B138" s="51"/>
-      <c r="C138" s="51"/>
+      <c r="B138" s="45"/>
+      <c r="C138" s="45"/>
       <c r="D138" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="19"/>
-      <c r="B139" s="51"/>
-      <c r="C139" s="51"/>
+      <c r="B139" s="45"/>
+      <c r="C139" s="45"/>
       <c r="D139" s="7" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="19"/>
-      <c r="B140" s="51"/>
-      <c r="C140" s="51"/>
+      <c r="B140" s="45"/>
+      <c r="C140" s="45"/>
       <c r="D140" s="7" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="19"/>
-      <c r="B141" s="51"/>
-      <c r="C141" s="51"/>
+      <c r="B141" s="45"/>
+      <c r="C141" s="45"/>
       <c r="D141" s="7" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="19"/>
-      <c r="B142" s="51"/>
-      <c r="C142" s="54">
+      <c r="B142" s="45"/>
+      <c r="C142" s="46">
         <v>3.1</v>
       </c>
       <c r="D142" s="7" t="s">
@@ -5918,122 +5925,122 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="19"/>
-      <c r="B143" s="51"/>
-      <c r="C143" s="54"/>
+      <c r="B143" s="45"/>
+      <c r="C143" s="46"/>
       <c r="D143" s="7" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="19"/>
-      <c r="B144" s="51"/>
-      <c r="C144" s="54"/>
+      <c r="B144" s="45"/>
+      <c r="C144" s="46"/>
       <c r="D144" s="7" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="19"/>
-      <c r="B145" s="51"/>
-      <c r="C145" s="54"/>
+      <c r="B145" s="45"/>
+      <c r="C145" s="46"/>
       <c r="D145" s="7" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="19"/>
-      <c r="B146" s="51"/>
-      <c r="C146" s="54"/>
+      <c r="B146" s="45"/>
+      <c r="C146" s="46"/>
       <c r="D146" s="7" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="19"/>
-      <c r="B147" s="51"/>
-      <c r="C147" s="54"/>
+      <c r="B147" s="45"/>
+      <c r="C147" s="46"/>
       <c r="D147" s="7" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="19"/>
-      <c r="B148" s="51"/>
-      <c r="C148" s="54"/>
+      <c r="B148" s="45"/>
+      <c r="C148" s="46"/>
       <c r="D148" s="7" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="19"/>
-      <c r="B149" s="51"/>
-      <c r="C149" s="54"/>
+      <c r="B149" s="45"/>
+      <c r="C149" s="46"/>
       <c r="D149" s="7" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="19"/>
-      <c r="B150" s="51"/>
-      <c r="C150" s="54"/>
+      <c r="B150" s="45"/>
+      <c r="C150" s="46"/>
       <c r="D150" s="7" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="19"/>
-      <c r="B151" s="51"/>
-      <c r="C151" s="54"/>
+      <c r="B151" s="45"/>
+      <c r="C151" s="46"/>
       <c r="D151" s="7" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="19"/>
-      <c r="B152" s="51"/>
-      <c r="C152" s="54"/>
+      <c r="B152" s="45"/>
+      <c r="C152" s="46"/>
       <c r="D152" s="7" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="19"/>
-      <c r="B153" s="51"/>
-      <c r="C153" s="54"/>
+      <c r="B153" s="45"/>
+      <c r="C153" s="46"/>
       <c r="D153" s="7" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="19"/>
-      <c r="B154" s="51"/>
-      <c r="C154" s="54"/>
+      <c r="B154" s="45"/>
+      <c r="C154" s="46"/>
       <c r="D154" s="7" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="19"/>
-      <c r="B155" s="51"/>
-      <c r="C155" s="54"/>
+      <c r="B155" s="45"/>
+      <c r="C155" s="46"/>
       <c r="D155" s="7" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="19"/>
-      <c r="B156" s="51"/>
-      <c r="C156" s="54"/>
+      <c r="B156" s="45"/>
+      <c r="C156" s="46"/>
       <c r="D156" s="7" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="20"/>
-      <c r="B157" s="51">
+      <c r="B157" s="45">
         <v>4</v>
       </c>
-      <c r="C157" s="51">
+      <c r="C157" s="45">
         <v>4.0999999999999996</v>
       </c>
       <c r="D157" s="7" t="s">
@@ -6042,32 +6049,32 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="19"/>
-      <c r="B158" s="51"/>
-      <c r="C158" s="51"/>
+      <c r="B158" s="45"/>
+      <c r="C158" s="45"/>
       <c r="D158" s="7" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="19"/>
-      <c r="B159" s="51"/>
-      <c r="C159" s="51"/>
+      <c r="B159" s="45"/>
+      <c r="C159" s="45"/>
       <c r="D159" s="7" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="19"/>
-      <c r="B160" s="51"/>
-      <c r="C160" s="51"/>
+      <c r="B160" s="45"/>
+      <c r="C160" s="45"/>
       <c r="D160" s="7" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="19"/>
-      <c r="B161" s="51"/>
-      <c r="C161" s="51">
+      <c r="B161" s="45"/>
+      <c r="C161" s="45">
         <v>4.2</v>
       </c>
       <c r="D161" s="7" t="s">
@@ -6076,56 +6083,56 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="19"/>
-      <c r="B162" s="51"/>
-      <c r="C162" s="51"/>
+      <c r="B162" s="45"/>
+      <c r="C162" s="45"/>
       <c r="D162" s="7" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="19"/>
-      <c r="B163" s="51"/>
-      <c r="C163" s="51"/>
+      <c r="B163" s="45"/>
+      <c r="C163" s="45"/>
       <c r="D163" s="7" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="19"/>
-      <c r="B164" s="51"/>
-      <c r="C164" s="51"/>
+      <c r="B164" s="45"/>
+      <c r="C164" s="45"/>
       <c r="D164" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="19"/>
-      <c r="B165" s="51"/>
-      <c r="C165" s="51"/>
+      <c r="B165" s="45"/>
+      <c r="C165" s="45"/>
       <c r="D165" s="7" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="19"/>
-      <c r="B166" s="51"/>
-      <c r="C166" s="51"/>
+      <c r="B166" s="45"/>
+      <c r="C166" s="45"/>
       <c r="D166" s="7" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="19"/>
-      <c r="B167" s="51"/>
-      <c r="C167" s="51"/>
+      <c r="B167" s="45"/>
+      <c r="C167" s="45"/>
       <c r="D167" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="19"/>
-      <c r="B168" s="51"/>
-      <c r="C168" s="51">
+      <c r="B168" s="45"/>
+      <c r="C168" s="45">
         <v>4.3</v>
       </c>
       <c r="D168" s="7" t="s">
@@ -6134,48 +6141,48 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="19"/>
-      <c r="B169" s="51"/>
-      <c r="C169" s="51"/>
+      <c r="B169" s="45"/>
+      <c r="C169" s="45"/>
       <c r="D169" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="19"/>
-      <c r="B170" s="51"/>
-      <c r="C170" s="51"/>
+      <c r="B170" s="45"/>
+      <c r="C170" s="45"/>
       <c r="D170" s="7" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="19"/>
-      <c r="B171" s="51"/>
-      <c r="C171" s="51"/>
+      <c r="B171" s="45"/>
+      <c r="C171" s="45"/>
       <c r="D171" s="7" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="19"/>
-      <c r="B172" s="51"/>
-      <c r="C172" s="51"/>
+      <c r="B172" s="45"/>
+      <c r="C172" s="45"/>
       <c r="D172" s="7" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="19"/>
-      <c r="B173" s="51"/>
-      <c r="C173" s="51"/>
+      <c r="B173" s="45"/>
+      <c r="C173" s="45"/>
       <c r="D173" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="19"/>
-      <c r="B174" s="51"/>
-      <c r="C174" s="51">
+      <c r="B174" s="45"/>
+      <c r="C174" s="45">
         <v>4.4000000000000004</v>
       </c>
       <c r="D174" s="7" t="s">
@@ -6184,63 +6191,98 @@
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="19"/>
-      <c r="B175" s="51"/>
-      <c r="C175" s="51"/>
+      <c r="B175" s="45"/>
+      <c r="C175" s="45"/>
       <c r="D175" s="7" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="19"/>
-      <c r="B176" s="51"/>
-      <c r="C176" s="51"/>
+      <c r="B176" s="45"/>
+      <c r="C176" s="45"/>
       <c r="D176" s="7" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" s="19"/>
-      <c r="B177" s="51"/>
-      <c r="C177" s="51"/>
+      <c r="B177" s="45"/>
+      <c r="C177" s="45"/>
       <c r="D177" s="7" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" s="19"/>
-      <c r="B178" s="51"/>
-      <c r="C178" s="51"/>
+      <c r="B178" s="45"/>
+      <c r="C178" s="45"/>
       <c r="D178" s="7" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="19"/>
-      <c r="B179" s="51"/>
-      <c r="C179" s="51"/>
+      <c r="B179" s="45"/>
+      <c r="C179" s="45"/>
       <c r="D179" s="7" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="180" spans="1:4">
       <c r="A180" s="19"/>
-      <c r="B180" s="51"/>
-      <c r="C180" s="51"/>
+      <c r="B180" s="45"/>
+      <c r="C180" s="45"/>
       <c r="D180" s="7" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="181" spans="1:4">
       <c r="A181" s="19"/>
-      <c r="B181" s="51"/>
-      <c r="C181" s="51"/>
+      <c r="B181" s="45"/>
+      <c r="C181" s="45"/>
       <c r="D181" s="7" t="s">
         <v>57</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J181" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A2:J181"/>
   <mergeCells count="51">
+    <mergeCell ref="F50:F58"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="F31:F37"/>
+    <mergeCell ref="F38:F45"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E50:E58"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="A3:A58"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="B26:B58"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E31:E37"/>
+    <mergeCell ref="C18:C25"/>
+    <mergeCell ref="G31:G37"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="E18:E25"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="F18:F25"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="E3:E11"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="F3:F11"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="C3:C11"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="C110:C115"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C31:C37"/>
+    <mergeCell ref="C38:C45"/>
+    <mergeCell ref="C50:C58"/>
     <mergeCell ref="C168:C173"/>
     <mergeCell ref="C174:C181"/>
     <mergeCell ref="B3:B25"/>
@@ -6257,41 +6299,6 @@
     <mergeCell ref="C77:C87"/>
     <mergeCell ref="C88:C100"/>
     <mergeCell ref="C101:C109"/>
-    <mergeCell ref="C110:C115"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C31:C37"/>
-    <mergeCell ref="C38:C45"/>
-    <mergeCell ref="C50:C58"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="E3:E11"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="F3:F11"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="C3:C11"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C15:C17"/>
-    <mergeCell ref="G31:G37"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="E18:E25"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="F18:F25"/>
-    <mergeCell ref="E50:E58"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="A3:A58"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="B26:B58"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E37"/>
-    <mergeCell ref="C18:C25"/>
-    <mergeCell ref="F50:F58"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="F31:F37"/>
-    <mergeCell ref="F38:F45"/>
-    <mergeCell ref="F46:F49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6300,32 +6307,32 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" style="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="15" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
     </row>
     <row r="2" spans="1:12" s="4" customFormat="1">
       <c r="A2" s="32" t="s">
@@ -6363,11 +6370,11 @@
       </c>
       <c r="L2" s="40"/>
     </row>
-    <row r="3" spans="1:12" ht="129.6">
-      <c r="A3" s="44">
+    <row r="3" spans="1:12" ht="135">
+      <c r="A3" s="53">
         <v>1</v>
       </c>
-      <c r="B3" s="44">
+      <c r="B3" s="53">
         <v>1</v>
       </c>
       <c r="C3" s="15">
@@ -6390,9 +6397,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="57.6">
-      <c r="A4" s="44"/>
-      <c r="B4" s="44"/>
+    <row r="4" spans="1:12" ht="60">
+      <c r="A4" s="53"/>
+      <c r="B4" s="53"/>
       <c r="C4" s="15">
         <v>1.2</v>
       </c>
@@ -6413,9 +6420,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="43.2">
-      <c r="A5" s="44"/>
-      <c r="B5" s="44"/>
+    <row r="5" spans="1:12" ht="45">
+      <c r="A5" s="53"/>
+      <c r="B5" s="53"/>
       <c r="C5" s="15">
         <v>1.3</v>
       </c>
@@ -6436,9 +6443,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="115.2">
-      <c r="A6" s="44"/>
-      <c r="B6" s="44"/>
+    <row r="6" spans="1:12" ht="120">
+      <c r="A6" s="53"/>
+      <c r="B6" s="53"/>
       <c r="C6" s="36">
         <v>1.4</v>
       </c>
@@ -6461,9 +6468,9 @@
       <c r="I6" s="38"/>
       <c r="J6" s="38"/>
     </row>
-    <row r="7" spans="1:12" ht="72">
-      <c r="A7" s="44"/>
-      <c r="B7" s="44">
+    <row r="7" spans="1:12" ht="90">
+      <c r="A7" s="53"/>
+      <c r="B7" s="53">
         <v>2</v>
       </c>
       <c r="C7" s="15">
@@ -6486,9 +6493,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="57.6">
-      <c r="A8" s="44"/>
-      <c r="B8" s="44"/>
+    <row r="8" spans="1:12" ht="60">
+      <c r="A8" s="53"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -6509,9 +6516,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="100.8">
-      <c r="A9" s="44"/>
-      <c r="B9" s="44"/>
+    <row r="9" spans="1:12" ht="105">
+      <c r="A9" s="53"/>
+      <c r="B9" s="53"/>
       <c r="C9" s="15">
         <v>2.2999999999999998</v>
       </c>
@@ -6526,15 +6533,15 @@
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>212</v>
+        <v>245</v>
       </c>
       <c r="H9" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="115.2">
-      <c r="A10" s="44"/>
-      <c r="B10" s="44"/>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="120">
+      <c r="A10" s="53"/>
+      <c r="B10" s="53"/>
       <c r="C10" s="15">
         <v>2.4</v>
       </c>
@@ -6555,9 +6562,9 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="100.8">
-      <c r="A11" s="44"/>
-      <c r="B11" s="44"/>
+    <row r="11" spans="1:12" ht="120">
+      <c r="A11" s="53"/>
+      <c r="B11" s="53"/>
       <c r="C11" s="15">
         <v>2.5</v>
       </c>
@@ -6575,12 +6582,12 @@
         <v>245</v>
       </c>
       <c r="H11" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="115.2">
-      <c r="A12" s="44"/>
-      <c r="B12" s="44"/>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="120">
+      <c r="A12" s="53"/>
+      <c r="B12" s="53"/>
       <c r="C12" s="15">
         <v>2.6</v>
       </c>
@@ -6601,9 +6608,9 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="158.4">
-      <c r="A13" s="44"/>
-      <c r="B13" s="44"/>
+    <row r="13" spans="1:12" ht="165">
+      <c r="A13" s="53"/>
+      <c r="B13" s="53"/>
       <c r="C13" s="36">
         <v>2.7</v>
       </c>
@@ -6626,7 +6633,7 @@
       <c r="I13" s="38"/>
       <c r="J13" s="38"/>
     </row>
-    <row r="14" spans="1:12" ht="144">
+    <row r="14" spans="1:12" ht="165">
       <c r="C14" s="41">
         <v>2.8</v>
       </c>
@@ -6666,11 +6673,11 @@
       <c r="I15" s="29"/>
       <c r="J15" s="31"/>
     </row>
-    <row r="16" spans="1:12" ht="86.4">
-      <c r="A16" s="45">
+    <row r="16" spans="1:12" ht="90">
+      <c r="A16" s="54">
         <v>2</v>
       </c>
-      <c r="B16" s="45">
+      <c r="B16" s="54">
         <v>3</v>
       </c>
       <c r="C16" s="15">
@@ -6680,9 +6687,9 @@
         <v>234</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="86.4">
-      <c r="A17" s="44"/>
-      <c r="B17" s="44"/>
+    <row r="17" spans="1:4" ht="90">
+      <c r="A17" s="53"/>
+      <c r="B17" s="53"/>
       <c r="C17" s="15">
         <v>3.2</v>
       </c>
@@ -6690,9 +6697,9 @@
         <v>266</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="86.4">
-      <c r="A18" s="44"/>
-      <c r="B18" s="44"/>
+    <row r="18" spans="1:4" ht="90">
+      <c r="A18" s="53"/>
+      <c r="B18" s="53"/>
       <c r="C18" s="15">
         <v>3.3</v>
       </c>
@@ -6700,9 +6707,9 @@
         <v>265</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="158.4">
-      <c r="A19" s="44"/>
-      <c r="B19" s="44"/>
+    <row r="19" spans="1:4" ht="165">
+      <c r="A19" s="53"/>
+      <c r="B19" s="53"/>
       <c r="C19" s="15">
         <v>3.4</v>
       </c>
@@ -6710,9 +6717,9 @@
         <v>235</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="100.8">
-      <c r="A20" s="44"/>
-      <c r="B20" s="44"/>
+    <row r="20" spans="1:4" ht="105">
+      <c r="A20" s="53"/>
+      <c r="B20" s="53"/>
       <c r="C20" s="15">
         <v>3.5</v>
       </c>
@@ -6720,9 +6727,9 @@
         <v>267</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="115.2">
-      <c r="A21" s="44"/>
-      <c r="B21" s="44"/>
+    <row r="21" spans="1:4" ht="120">
+      <c r="A21" s="53"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="15">
         <v>3.6</v>
       </c>
@@ -6731,8 +6738,8 @@
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="44"/>
-      <c r="B22" s="44"/>
+      <c r="A22" s="53"/>
+      <c r="B22" s="53"/>
       <c r="C22" s="15">
         <v>3.7</v>
       </c>
@@ -6740,9 +6747,9 @@
         <v>268</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="86.4">
-      <c r="A23" s="44"/>
-      <c r="B23" s="44"/>
+    <row r="23" spans="1:4" ht="90">
+      <c r="A23" s="53"/>
+      <c r="B23" s="53"/>
       <c r="C23" s="15">
         <v>3.8</v>
       </c>
@@ -6750,9 +6757,9 @@
         <v>236</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="158.4">
-      <c r="A24" s="44"/>
-      <c r="B24" s="44"/>
+    <row r="24" spans="1:4" ht="165">
+      <c r="A24" s="53"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="15">
         <v>3.9</v>
       </c>
@@ -6760,9 +6767,9 @@
         <v>237</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="144">
-      <c r="A25" s="44"/>
-      <c r="B25" s="44"/>
+    <row r="25" spans="1:4" ht="150">
+      <c r="A25" s="53"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="35">
         <v>3.1</v>
       </c>
@@ -6770,9 +6777,9 @@
         <v>238</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="72">
-      <c r="A26" s="44"/>
-      <c r="B26" s="44"/>
+    <row r="26" spans="1:4" ht="75">
+      <c r="A26" s="53"/>
+      <c r="B26" s="53"/>
       <c r="C26" s="15">
         <v>3.11</v>
       </c>
@@ -6780,9 +6787,9 @@
         <v>239</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="216">
-      <c r="A27" s="44"/>
-      <c r="B27" s="44"/>
+    <row r="27" spans="1:4" ht="225">
+      <c r="A27" s="53"/>
+      <c r="B27" s="53"/>
       <c r="C27" s="35">
         <v>3.12</v>
       </c>
@@ -6790,9 +6797,9 @@
         <v>240</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="57.6">
-      <c r="A28" s="44"/>
-      <c r="B28" s="44">
+    <row r="28" spans="1:4" ht="60">
+      <c r="A28" s="53"/>
+      <c r="B28" s="53">
         <v>4</v>
       </c>
       <c r="C28" s="15">
@@ -6802,9 +6809,9 @@
         <v>241</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="100.8">
-      <c r="A29" s="44"/>
-      <c r="B29" s="44"/>
+    <row r="29" spans="1:4" ht="105">
+      <c r="A29" s="53"/>
+      <c r="B29" s="53"/>
       <c r="C29" s="15">
         <v>4.2</v>
       </c>
@@ -6812,9 +6819,9 @@
         <v>242</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="86.4">
-      <c r="A30" s="44"/>
-      <c r="B30" s="44"/>
+    <row r="30" spans="1:4" ht="90">
+      <c r="A30" s="53"/>
+      <c r="B30" s="53"/>
       <c r="C30" s="15">
         <v>4.3</v>
       </c>
@@ -6822,9 +6829,9 @@
         <v>243</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="115.2">
-      <c r="A31" s="44"/>
-      <c r="B31" s="44"/>
+    <row r="31" spans="1:4" ht="120">
+      <c r="A31" s="53"/>
+      <c r="B31" s="53"/>
       <c r="C31" s="15">
         <v>4.4000000000000004</v>
       </c>
@@ -6849,17 +6856,17 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.88671875" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="57.6">
+    <row r="1" spans="1:5" ht="60">
       <c r="A1" s="22" t="s">
         <v>214</v>
       </c>
@@ -7057,9 +7064,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="55" t="s">

</xml_diff>

<commit_message>
async & create_session API
rewired the backend back to async workflow ; decoupled image validation and image analysis api ; added POST /api/v1/sessions for session creation
</commit_message>
<xml_diff>
--- a/project_plan.xlsx
+++ b/project_plan.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B4D0E2-045B-45F8-AF15-C64E3B4E5798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB83E566-FA09-483D-8770-FD55689CD7DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2993,15 +2993,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3009,7 +3000,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4686,632 +4686,632 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="54">
+      <c r="A3" s="51">
         <v>1</v>
       </c>
-      <c r="B3" s="49">
+      <c r="B3" s="52">
         <v>1</v>
       </c>
-      <c r="C3" s="49">
+      <c r="C3" s="52">
         <v>1.1000000000000001</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="52" t="s">
+      <c r="E3" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="52" cm="1">
+      <c r="F3" s="49" cm="1">
         <f t="array" ref="F3">_xlfn.SWITCH(E3,"XS",1,"S",2,"M",3,"L",5,"XL",8,"XXL",13,"XXXL",21,"")</f>
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="54"/>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
+      <c r="A4" s="51"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
       <c r="D4" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="54"/>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
+      <c r="A5" s="51"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
       <c r="D5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="54"/>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
+      <c r="A6" s="51"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="52"/>
       <c r="D6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="54"/>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
+      <c r="A7" s="51"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
       <c r="D7" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="54"/>
-      <c r="B8" s="49"/>
-      <c r="C8" s="49"/>
+      <c r="A8" s="51"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="52"/>
       <c r="D8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="54"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
+      <c r="A9" s="51"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="52"/>
       <c r="D9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="54"/>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="52"/>
       <c r="D10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="52"/>
-      <c r="F10" s="52"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="54"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="49"/>
+      <c r="A11" s="51"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
       <c r="D11" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="54"/>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49">
+      <c r="A12" s="51"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52">
         <v>1.2</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="52" t="s">
+      <c r="E12" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="52" cm="1">
+      <c r="F12" s="49" cm="1">
         <f t="array" ref="F12">_xlfn.SWITCH(E3,"XS",1,"S",2,"M",3,"L",5,"XL",8,"XXL",13,"XXXL",21,"")</f>
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="54"/>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
       <c r="D13" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="52"/>
-      <c r="F13" s="52"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="54"/>
-      <c r="B14" s="49"/>
-      <c r="C14" s="49"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
       <c r="D14" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="54"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49">
+      <c r="A15" s="51"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="52">
         <v>1.3</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="52" t="s">
+      <c r="E15" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="52"/>
+      <c r="F15" s="49"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="54"/>
-      <c r="B16" s="49"/>
-      <c r="C16" s="49"/>
+      <c r="A16" s="51"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="52"/>
       <c r="D16" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="54"/>
-      <c r="B17" s="49"/>
-      <c r="C17" s="49"/>
+      <c r="A17" s="51"/>
+      <c r="B17" s="52"/>
+      <c r="C17" s="52"/>
       <c r="D17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="52"/>
-      <c r="F17" s="52"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="54"/>
-      <c r="B18" s="49"/>
-      <c r="C18" s="49">
+      <c r="A18" s="51"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="52">
         <v>1.4</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="52" t="s">
+      <c r="E18" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="52"/>
+      <c r="F18" s="49"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="54"/>
-      <c r="B19" s="49"/>
-      <c r="C19" s="49"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="52"/>
       <c r="D19" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="54"/>
-      <c r="B20" s="49"/>
-      <c r="C20" s="49"/>
+      <c r="A20" s="51"/>
+      <c r="B20" s="52"/>
+      <c r="C20" s="52"/>
       <c r="D20" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="54"/>
-      <c r="B21" s="49"/>
-      <c r="C21" s="49"/>
+      <c r="A21" s="51"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
       <c r="D21" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="54"/>
-      <c r="B22" s="49"/>
-      <c r="C22" s="49"/>
+      <c r="A22" s="51"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
       <c r="D22" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="54"/>
-      <c r="B23" s="49"/>
-      <c r="C23" s="49"/>
+      <c r="A23" s="51"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="52"/>
       <c r="D23" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="54"/>
-      <c r="B24" s="49"/>
-      <c r="C24" s="49"/>
+      <c r="A24" s="51"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
       <c r="D24" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="54"/>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
       <c r="D25" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="54"/>
-      <c r="B26" s="55">
+      <c r="A26" s="51"/>
+      <c r="B26" s="53">
         <v>2</v>
       </c>
-      <c r="C26" s="49">
+      <c r="C26" s="52">
         <v>2.1</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E26" s="53" t="s">
+      <c r="E26" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="52"/>
+      <c r="F26" s="49"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="54"/>
-      <c r="B27" s="55"/>
-      <c r="C27" s="49"/>
+      <c r="A27" s="51"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="52"/>
       <c r="D27" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="53"/>
-      <c r="F27" s="52"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="49"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="54"/>
-      <c r="B28" s="55"/>
-      <c r="C28" s="49"/>
+      <c r="A28" s="51"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="52"/>
       <c r="D28" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="E28" s="53"/>
-      <c r="F28" s="52"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="49"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="54"/>
-      <c r="B29" s="55"/>
-      <c r="C29" s="51">
+      <c r="A29" s="51"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="54">
         <v>2.2000000000000002</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="52" t="s">
+      <c r="E29" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="52"/>
+      <c r="F29" s="49"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="54"/>
-      <c r="B30" s="55"/>
-      <c r="C30" s="51"/>
+      <c r="A30" s="51"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="54"/>
       <c r="D30" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E30" s="52"/>
-      <c r="F30" s="52"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="54"/>
-      <c r="B31" s="55"/>
-      <c r="C31" s="49">
+      <c r="A31" s="51"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="52">
         <v>2.2999999999999998</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E31" s="52" t="s">
+      <c r="E31" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="F31" s="52"/>
-      <c r="G31" s="52" t="s">
+      <c r="F31" s="49"/>
+      <c r="G31" s="49" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="54"/>
-      <c r="B32" s="55"/>
-      <c r="C32" s="49"/>
+      <c r="A32" s="51"/>
+      <c r="B32" s="53"/>
+      <c r="C32" s="52"/>
       <c r="D32" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="54"/>
-      <c r="B33" s="55"/>
-      <c r="C33" s="49"/>
+      <c r="A33" s="51"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="52"/>
       <c r="D33" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="54"/>
-      <c r="B34" s="55"/>
-      <c r="C34" s="49"/>
+      <c r="A34" s="51"/>
+      <c r="B34" s="53"/>
+      <c r="C34" s="52"/>
       <c r="D34" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="49"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="54"/>
-      <c r="B35" s="55"/>
-      <c r="C35" s="49"/>
+      <c r="A35" s="51"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="52"/>
       <c r="D35" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="54"/>
-      <c r="B36" s="55"/>
-      <c r="C36" s="49"/>
+      <c r="A36" s="51"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="52"/>
       <c r="D36" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E36" s="52"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="52"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="54"/>
-      <c r="B37" s="55"/>
-      <c r="C37" s="49"/>
+      <c r="A37" s="51"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="52"/>
       <c r="D37" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="49"/>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="54"/>
-      <c r="B38" s="55"/>
-      <c r="C38" s="49">
+      <c r="A38" s="51"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="52">
         <v>2.4</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="52" t="s">
+      <c r="E38" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="52"/>
+      <c r="F38" s="49"/>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="54"/>
-      <c r="B39" s="55"/>
-      <c r="C39" s="49"/>
+      <c r="A39" s="51"/>
+      <c r="B39" s="53"/>
+      <c r="C39" s="52"/>
       <c r="D39" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="54"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="49"/>
+      <c r="A40" s="51"/>
+      <c r="B40" s="53"/>
+      <c r="C40" s="52"/>
       <c r="D40" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="54"/>
-      <c r="B41" s="55"/>
-      <c r="C41" s="49"/>
+      <c r="A41" s="51"/>
+      <c r="B41" s="53"/>
+      <c r="C41" s="52"/>
       <c r="D41" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="54"/>
-      <c r="B42" s="55"/>
-      <c r="C42" s="49"/>
+      <c r="A42" s="51"/>
+      <c r="B42" s="53"/>
+      <c r="C42" s="52"/>
       <c r="D42" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E42" s="52"/>
-      <c r="F42" s="52"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="54"/>
-      <c r="B43" s="55"/>
-      <c r="C43" s="49"/>
+      <c r="A43" s="51"/>
+      <c r="B43" s="53"/>
+      <c r="C43" s="52"/>
       <c r="D43" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="52"/>
-      <c r="F43" s="52"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="54"/>
-      <c r="B44" s="55"/>
-      <c r="C44" s="49"/>
+      <c r="A44" s="51"/>
+      <c r="B44" s="53"/>
+      <c r="C44" s="52"/>
       <c r="D44" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="E44" s="52"/>
-      <c r="F44" s="52"/>
+      <c r="E44" s="49"/>
+      <c r="F44" s="49"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="54"/>
-      <c r="B45" s="55"/>
-      <c r="C45" s="49"/>
+      <c r="A45" s="51"/>
+      <c r="B45" s="53"/>
+      <c r="C45" s="52"/>
       <c r="D45" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E45" s="52"/>
-      <c r="F45" s="52"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="54"/>
-      <c r="B46" s="55"/>
-      <c r="C46" s="49">
+      <c r="A46" s="51"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="52">
         <v>2.5</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E46" s="53" t="s">
+      <c r="E46" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="F46" s="52"/>
+      <c r="F46" s="49"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="54"/>
-      <c r="B47" s="55"/>
-      <c r="C47" s="49"/>
+      <c r="A47" s="51"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="52"/>
       <c r="D47" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E47" s="53"/>
-      <c r="F47" s="52"/>
+      <c r="E47" s="50"/>
+      <c r="F47" s="49"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="54"/>
-      <c r="B48" s="55"/>
-      <c r="C48" s="49"/>
+      <c r="A48" s="51"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="52"/>
       <c r="D48" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E48" s="53"/>
-      <c r="F48" s="52"/>
+      <c r="E48" s="50"/>
+      <c r="F48" s="49"/>
     </row>
     <row r="49" spans="1:6">
-      <c r="A49" s="54"/>
-      <c r="B49" s="55"/>
-      <c r="C49" s="49"/>
+      <c r="A49" s="51"/>
+      <c r="B49" s="53"/>
+      <c r="C49" s="52"/>
       <c r="D49" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E49" s="53"/>
-      <c r="F49" s="52"/>
+      <c r="E49" s="50"/>
+      <c r="F49" s="49"/>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="54"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="49">
+      <c r="A50" s="51"/>
+      <c r="B50" s="53"/>
+      <c r="C50" s="52">
         <v>2.7</v>
       </c>
       <c r="D50" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E50" s="52" t="s">
+      <c r="E50" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="F50" s="52"/>
+      <c r="F50" s="49"/>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="54"/>
-      <c r="B51" s="55"/>
-      <c r="C51" s="49"/>
+      <c r="A51" s="51"/>
+      <c r="B51" s="53"/>
+      <c r="C51" s="52"/>
       <c r="D51" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="54"/>
-      <c r="B52" s="55"/>
-      <c r="C52" s="49"/>
+      <c r="A52" s="51"/>
+      <c r="B52" s="53"/>
+      <c r="C52" s="52"/>
       <c r="D52" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E52" s="52"/>
-      <c r="F52" s="52"/>
+      <c r="E52" s="49"/>
+      <c r="F52" s="49"/>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="54"/>
-      <c r="B53" s="55"/>
-      <c r="C53" s="49"/>
+      <c r="A53" s="51"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="52"/>
       <c r="D53" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E53" s="52"/>
-      <c r="F53" s="52"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
     </row>
     <row r="54" spans="1:6">
-      <c r="A54" s="54"/>
-      <c r="B54" s="55"/>
-      <c r="C54" s="49"/>
+      <c r="A54" s="51"/>
+      <c r="B54" s="53"/>
+      <c r="C54" s="52"/>
       <c r="D54" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E54" s="52"/>
-      <c r="F54" s="52"/>
+      <c r="E54" s="49"/>
+      <c r="F54" s="49"/>
     </row>
     <row r="55" spans="1:6">
-      <c r="A55" s="54"/>
-      <c r="B55" s="55"/>
-      <c r="C55" s="49"/>
+      <c r="A55" s="51"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="52"/>
       <c r="D55" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
+      <c r="E55" s="49"/>
+      <c r="F55" s="49"/>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="54"/>
-      <c r="B56" s="55"/>
-      <c r="C56" s="49"/>
+      <c r="A56" s="51"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="52"/>
       <c r="D56" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
+      <c r="E56" s="49"/>
+      <c r="F56" s="49"/>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="54"/>
-      <c r="B57" s="55"/>
-      <c r="C57" s="49"/>
+      <c r="A57" s="51"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="52"/>
       <c r="D57" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
+      <c r="E57" s="49"/>
+      <c r="F57" s="49"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="54"/>
-      <c r="B58" s="55"/>
-      <c r="C58" s="49"/>
+      <c r="A58" s="51"/>
+      <c r="B58" s="53"/>
+      <c r="C58" s="52"/>
       <c r="D58" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="20"/>
-      <c r="B59" s="49">
+      <c r="B59" s="52">
         <v>3</v>
       </c>
-      <c r="C59" s="49">
+      <c r="C59" s="52">
         <v>3.1</v>
       </c>
       <c r="D59" s="7" t="s">
@@ -5320,48 +5320,48 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="19"/>
-      <c r="B60" s="49"/>
-      <c r="C60" s="49"/>
+      <c r="B60" s="52"/>
+      <c r="C60" s="52"/>
       <c r="D60" s="7" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="19"/>
-      <c r="B61" s="49"/>
-      <c r="C61" s="49"/>
+      <c r="B61" s="52"/>
+      <c r="C61" s="52"/>
       <c r="D61" s="7" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="19"/>
-      <c r="B62" s="49"/>
-      <c r="C62" s="49"/>
+      <c r="B62" s="52"/>
+      <c r="C62" s="52"/>
       <c r="D62" s="7" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="19"/>
-      <c r="B63" s="49"/>
-      <c r="C63" s="49"/>
+      <c r="B63" s="52"/>
+      <c r="C63" s="52"/>
       <c r="D63" s="7" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="19"/>
-      <c r="B64" s="49"/>
-      <c r="C64" s="49"/>
+      <c r="B64" s="52"/>
+      <c r="C64" s="52"/>
       <c r="D64" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="19"/>
-      <c r="B65" s="49"/>
-      <c r="C65" s="49">
+      <c r="B65" s="52"/>
+      <c r="C65" s="52">
         <v>3.2</v>
       </c>
       <c r="D65" s="7" t="s">
@@ -5370,96 +5370,96 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="19"/>
-      <c r="B66" s="49"/>
-      <c r="C66" s="49"/>
+      <c r="B66" s="52"/>
+      <c r="C66" s="52"/>
       <c r="D66" s="7" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="19"/>
-      <c r="B67" s="49"/>
-      <c r="C67" s="49"/>
+      <c r="B67" s="52"/>
+      <c r="C67" s="52"/>
       <c r="D67" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="19"/>
-      <c r="B68" s="49"/>
-      <c r="C68" s="49"/>
+      <c r="B68" s="52"/>
+      <c r="C68" s="52"/>
       <c r="D68" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="19"/>
-      <c r="B69" s="49"/>
-      <c r="C69" s="49"/>
+      <c r="B69" s="52"/>
+      <c r="C69" s="52"/>
       <c r="D69" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="19"/>
-      <c r="B70" s="49"/>
-      <c r="C70" s="49"/>
+      <c r="B70" s="52"/>
+      <c r="C70" s="52"/>
       <c r="D70" s="7" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="19"/>
-      <c r="B71" s="49"/>
-      <c r="C71" s="49"/>
+      <c r="B71" s="52"/>
+      <c r="C71" s="52"/>
       <c r="D71" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="19"/>
-      <c r="B72" s="49"/>
-      <c r="C72" s="49"/>
+      <c r="B72" s="52"/>
+      <c r="C72" s="52"/>
       <c r="D72" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="19"/>
-      <c r="B73" s="49"/>
-      <c r="C73" s="49"/>
+      <c r="B73" s="52"/>
+      <c r="C73" s="52"/>
       <c r="D73" s="7" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="19"/>
-      <c r="B74" s="49"/>
-      <c r="C74" s="49"/>
+      <c r="B74" s="52"/>
+      <c r="C74" s="52"/>
       <c r="D74" s="7" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="19"/>
-      <c r="B75" s="49"/>
-      <c r="C75" s="49"/>
+      <c r="B75" s="52"/>
+      <c r="C75" s="52"/>
       <c r="D75" s="7" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="19"/>
-      <c r="B76" s="49"/>
-      <c r="C76" s="49"/>
+      <c r="B76" s="52"/>
+      <c r="C76" s="52"/>
       <c r="D76" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="19"/>
-      <c r="B77" s="49"/>
-      <c r="C77" s="49">
+      <c r="B77" s="52"/>
+      <c r="C77" s="52">
         <v>3.3</v>
       </c>
       <c r="D77" s="7" t="s">
@@ -5468,88 +5468,88 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="19"/>
-      <c r="B78" s="49"/>
-      <c r="C78" s="49"/>
+      <c r="B78" s="52"/>
+      <c r="C78" s="52"/>
       <c r="D78" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="19"/>
-      <c r="B79" s="49"/>
-      <c r="C79" s="49"/>
+      <c r="B79" s="52"/>
+      <c r="C79" s="52"/>
       <c r="D79" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="19"/>
-      <c r="B80" s="49"/>
-      <c r="C80" s="49"/>
+      <c r="B80" s="52"/>
+      <c r="C80" s="52"/>
       <c r="D80" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="19"/>
-      <c r="B81" s="49"/>
-      <c r="C81" s="49"/>
+      <c r="B81" s="52"/>
+      <c r="C81" s="52"/>
       <c r="D81" s="7" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="19"/>
-      <c r="B82" s="49"/>
-      <c r="C82" s="49"/>
+      <c r="B82" s="52"/>
+      <c r="C82" s="52"/>
       <c r="D82" s="7" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="19"/>
-      <c r="B83" s="49"/>
-      <c r="C83" s="49"/>
+      <c r="B83" s="52"/>
+      <c r="C83" s="52"/>
       <c r="D83" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="19"/>
-      <c r="B84" s="49"/>
-      <c r="C84" s="49"/>
+      <c r="B84" s="52"/>
+      <c r="C84" s="52"/>
       <c r="D84" s="7" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="19"/>
-      <c r="B85" s="49"/>
-      <c r="C85" s="49"/>
+      <c r="B85" s="52"/>
+      <c r="C85" s="52"/>
       <c r="D85" s="7" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="19"/>
-      <c r="B86" s="49"/>
-      <c r="C86" s="49"/>
+      <c r="B86" s="52"/>
+      <c r="C86" s="52"/>
       <c r="D86" s="7" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="19"/>
-      <c r="B87" s="49"/>
-      <c r="C87" s="49"/>
+      <c r="B87" s="52"/>
+      <c r="C87" s="52"/>
       <c r="D87" s="7" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="19"/>
-      <c r="B88" s="49"/>
-      <c r="C88" s="49">
+      <c r="B88" s="52"/>
+      <c r="C88" s="52">
         <v>3.4</v>
       </c>
       <c r="D88" s="15" t="s">
@@ -5558,104 +5558,104 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="19"/>
-      <c r="B89" s="49"/>
-      <c r="C89" s="49"/>
+      <c r="B89" s="52"/>
+      <c r="C89" s="52"/>
       <c r="D89" s="7" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="19"/>
-      <c r="B90" s="49"/>
-      <c r="C90" s="49"/>
+      <c r="B90" s="52"/>
+      <c r="C90" s="52"/>
       <c r="D90" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="19"/>
-      <c r="B91" s="49"/>
-      <c r="C91" s="49"/>
+      <c r="B91" s="52"/>
+      <c r="C91" s="52"/>
       <c r="D91" s="7" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="19"/>
-      <c r="B92" s="49"/>
-      <c r="C92" s="49"/>
+      <c r="B92" s="52"/>
+      <c r="C92" s="52"/>
       <c r="D92" s="7" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="19"/>
-      <c r="B93" s="49"/>
-      <c r="C93" s="49"/>
+      <c r="B93" s="52"/>
+      <c r="C93" s="52"/>
       <c r="D93" s="7" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="19"/>
-      <c r="B94" s="49"/>
-      <c r="C94" s="49"/>
+      <c r="B94" s="52"/>
+      <c r="C94" s="52"/>
       <c r="D94" s="7" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="19"/>
-      <c r="B95" s="49"/>
-      <c r="C95" s="49"/>
+      <c r="B95" s="52"/>
+      <c r="C95" s="52"/>
       <c r="D95" s="7" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="19"/>
-      <c r="B96" s="49"/>
-      <c r="C96" s="49"/>
+      <c r="B96" s="52"/>
+      <c r="C96" s="52"/>
       <c r="D96" s="7" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="19"/>
-      <c r="B97" s="49"/>
-      <c r="C97" s="49"/>
+      <c r="B97" s="52"/>
+      <c r="C97" s="52"/>
       <c r="D97" s="7" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="19"/>
-      <c r="B98" s="49"/>
-      <c r="C98" s="49"/>
+      <c r="B98" s="52"/>
+      <c r="C98" s="52"/>
       <c r="D98" s="7" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="19"/>
-      <c r="B99" s="49"/>
-      <c r="C99" s="49"/>
+      <c r="B99" s="52"/>
+      <c r="C99" s="52"/>
       <c r="D99" s="7" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="19"/>
-      <c r="B100" s="49"/>
-      <c r="C100" s="49"/>
+      <c r="B100" s="52"/>
+      <c r="C100" s="52"/>
       <c r="D100" s="7" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="19"/>
-      <c r="B101" s="49"/>
-      <c r="C101" s="49">
+      <c r="B101" s="52"/>
+      <c r="C101" s="52">
         <v>3.5</v>
       </c>
       <c r="D101" s="11" t="s">
@@ -5664,72 +5664,72 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="19"/>
-      <c r="B102" s="49"/>
-      <c r="C102" s="49"/>
+      <c r="B102" s="52"/>
+      <c r="C102" s="52"/>
       <c r="D102" s="7" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="19"/>
-      <c r="B103" s="49"/>
-      <c r="C103" s="49"/>
+      <c r="B103" s="52"/>
+      <c r="C103" s="52"/>
       <c r="D103" s="7" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="19"/>
-      <c r="B104" s="49"/>
-      <c r="C104" s="49"/>
+      <c r="B104" s="52"/>
+      <c r="C104" s="52"/>
       <c r="D104" s="7" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="19"/>
-      <c r="B105" s="49"/>
-      <c r="C105" s="49"/>
+      <c r="B105" s="52"/>
+      <c r="C105" s="52"/>
       <c r="D105" s="7" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="19"/>
-      <c r="B106" s="49"/>
-      <c r="C106" s="49"/>
+      <c r="B106" s="52"/>
+      <c r="C106" s="52"/>
       <c r="D106" s="7" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="19"/>
-      <c r="B107" s="49"/>
-      <c r="C107" s="49"/>
+      <c r="B107" s="52"/>
+      <c r="C107" s="52"/>
       <c r="D107" s="7" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="19"/>
-      <c r="B108" s="49"/>
-      <c r="C108" s="49"/>
+      <c r="B108" s="52"/>
+      <c r="C108" s="52"/>
       <c r="D108" s="7" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="19"/>
-      <c r="B109" s="49"/>
-      <c r="C109" s="49"/>
+      <c r="B109" s="52"/>
+      <c r="C109" s="52"/>
       <c r="D109" s="7" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="19"/>
-      <c r="B110" s="49"/>
-      <c r="C110" s="49">
+      <c r="B110" s="52"/>
+      <c r="C110" s="52">
         <v>3.6</v>
       </c>
       <c r="D110" s="7" t="s">
@@ -5738,48 +5738,48 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="19"/>
-      <c r="B111" s="49"/>
-      <c r="C111" s="49"/>
+      <c r="B111" s="52"/>
+      <c r="C111" s="52"/>
       <c r="D111" s="7" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="19"/>
-      <c r="B112" s="49"/>
-      <c r="C112" s="49"/>
+      <c r="B112" s="52"/>
+      <c r="C112" s="52"/>
       <c r="D112" s="7" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="19"/>
-      <c r="B113" s="49"/>
-      <c r="C113" s="49"/>
+      <c r="B113" s="52"/>
+      <c r="C113" s="52"/>
       <c r="D113" s="7" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="19"/>
-      <c r="B114" s="49"/>
-      <c r="C114" s="49"/>
+      <c r="B114" s="52"/>
+      <c r="C114" s="52"/>
       <c r="D114" s="7" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="19"/>
-      <c r="B115" s="49"/>
-      <c r="C115" s="49"/>
+      <c r="B115" s="52"/>
+      <c r="C115" s="52"/>
       <c r="D115" s="7" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="19"/>
-      <c r="B116" s="49"/>
-      <c r="C116" s="49">
+      <c r="B116" s="52"/>
+      <c r="C116" s="52">
         <v>3.7</v>
       </c>
       <c r="D116" s="7" t="s">
@@ -5788,88 +5788,88 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="19"/>
-      <c r="B117" s="49"/>
-      <c r="C117" s="49"/>
+      <c r="B117" s="52"/>
+      <c r="C117" s="52"/>
       <c r="D117" s="7" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="19"/>
-      <c r="B118" s="49"/>
-      <c r="C118" s="49"/>
+      <c r="B118" s="52"/>
+      <c r="C118" s="52"/>
       <c r="D118" s="7" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="19"/>
-      <c r="B119" s="49"/>
-      <c r="C119" s="49"/>
+      <c r="B119" s="52"/>
+      <c r="C119" s="52"/>
       <c r="D119" s="7" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="19"/>
-      <c r="B120" s="49"/>
-      <c r="C120" s="49"/>
+      <c r="B120" s="52"/>
+      <c r="C120" s="52"/>
       <c r="D120" s="7" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="19"/>
-      <c r="B121" s="49"/>
-      <c r="C121" s="49"/>
+      <c r="B121" s="52"/>
+      <c r="C121" s="52"/>
       <c r="D121" s="7" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="19"/>
-      <c r="B122" s="49"/>
-      <c r="C122" s="49"/>
+      <c r="B122" s="52"/>
+      <c r="C122" s="52"/>
       <c r="D122" s="7" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="19"/>
-      <c r="B123" s="49"/>
-      <c r="C123" s="49"/>
+      <c r="B123" s="52"/>
+      <c r="C123" s="52"/>
       <c r="D123" s="7" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="19"/>
-      <c r="B124" s="49"/>
-      <c r="C124" s="49"/>
+      <c r="B124" s="52"/>
+      <c r="C124" s="52"/>
       <c r="D124" s="7" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="19"/>
-      <c r="B125" s="49"/>
-      <c r="C125" s="49"/>
+      <c r="B125" s="52"/>
+      <c r="C125" s="52"/>
       <c r="D125" s="7" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="19"/>
-      <c r="B126" s="49"/>
-      <c r="C126" s="49"/>
+      <c r="B126" s="52"/>
+      <c r="C126" s="52"/>
       <c r="D126" s="7" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="19"/>
-      <c r="B127" s="49"/>
-      <c r="C127" s="49">
+      <c r="B127" s="52"/>
+      <c r="C127" s="52">
         <v>3.8</v>
       </c>
       <c r="D127" s="7" t="s">
@@ -5878,80 +5878,80 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="19"/>
-      <c r="B128" s="49"/>
-      <c r="C128" s="49"/>
+      <c r="B128" s="52"/>
+      <c r="C128" s="52"/>
       <c r="D128" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="19"/>
-      <c r="B129" s="49"/>
-      <c r="C129" s="49"/>
+      <c r="B129" s="52"/>
+      <c r="C129" s="52"/>
       <c r="D129" s="7" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="19"/>
-      <c r="B130" s="49"/>
-      <c r="C130" s="49"/>
+      <c r="B130" s="52"/>
+      <c r="C130" s="52"/>
       <c r="D130" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="19"/>
-      <c r="B131" s="49"/>
-      <c r="C131" s="49"/>
+      <c r="B131" s="52"/>
+      <c r="C131" s="52"/>
       <c r="D131" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="19"/>
-      <c r="B132" s="49"/>
-      <c r="C132" s="49"/>
+      <c r="B132" s="52"/>
+      <c r="C132" s="52"/>
       <c r="D132" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="19"/>
-      <c r="B133" s="49"/>
-      <c r="C133" s="49"/>
+      <c r="B133" s="52"/>
+      <c r="C133" s="52"/>
       <c r="D133" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="19"/>
-      <c r="B134" s="49"/>
-      <c r="C134" s="49"/>
+      <c r="B134" s="52"/>
+      <c r="C134" s="52"/>
       <c r="D134" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="19"/>
-      <c r="B135" s="49"/>
-      <c r="C135" s="49"/>
+      <c r="B135" s="52"/>
+      <c r="C135" s="52"/>
       <c r="D135" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="19"/>
-      <c r="B136" s="49"/>
-      <c r="C136" s="49"/>
+      <c r="B136" s="52"/>
+      <c r="C136" s="52"/>
       <c r="D136" s="7" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="19"/>
-      <c r="B137" s="49"/>
-      <c r="C137" s="49">
+      <c r="B137" s="52"/>
+      <c r="C137" s="52">
         <v>3.9</v>
       </c>
       <c r="D137" s="7" t="s">
@@ -5960,40 +5960,40 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="19"/>
-      <c r="B138" s="49"/>
-      <c r="C138" s="49"/>
+      <c r="B138" s="52"/>
+      <c r="C138" s="52"/>
       <c r="D138" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="19"/>
-      <c r="B139" s="49"/>
-      <c r="C139" s="49"/>
+      <c r="B139" s="52"/>
+      <c r="C139" s="52"/>
       <c r="D139" s="7" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="19"/>
-      <c r="B140" s="49"/>
-      <c r="C140" s="49"/>
+      <c r="B140" s="52"/>
+      <c r="C140" s="52"/>
       <c r="D140" s="7" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="19"/>
-      <c r="B141" s="49"/>
-      <c r="C141" s="49"/>
+      <c r="B141" s="52"/>
+      <c r="C141" s="52"/>
       <c r="D141" s="7" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="19"/>
-      <c r="B142" s="49"/>
-      <c r="C142" s="50">
+      <c r="B142" s="52"/>
+      <c r="C142" s="55">
         <v>3.1</v>
       </c>
       <c r="D142" s="7" t="s">
@@ -6002,122 +6002,122 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="19"/>
-      <c r="B143" s="49"/>
-      <c r="C143" s="50"/>
+      <c r="B143" s="52"/>
+      <c r="C143" s="55"/>
       <c r="D143" s="7" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="19"/>
-      <c r="B144" s="49"/>
-      <c r="C144" s="50"/>
+      <c r="B144" s="52"/>
+      <c r="C144" s="55"/>
       <c r="D144" s="7" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="19"/>
-      <c r="B145" s="49"/>
-      <c r="C145" s="50"/>
+      <c r="B145" s="52"/>
+      <c r="C145" s="55"/>
       <c r="D145" s="7" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="19"/>
-      <c r="B146" s="49"/>
-      <c r="C146" s="50"/>
+      <c r="B146" s="52"/>
+      <c r="C146" s="55"/>
       <c r="D146" s="7" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="19"/>
-      <c r="B147" s="49"/>
-      <c r="C147" s="50"/>
+      <c r="B147" s="52"/>
+      <c r="C147" s="55"/>
       <c r="D147" s="7" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="19"/>
-      <c r="B148" s="49"/>
-      <c r="C148" s="50"/>
+      <c r="B148" s="52"/>
+      <c r="C148" s="55"/>
       <c r="D148" s="7" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="19"/>
-      <c r="B149" s="49"/>
-      <c r="C149" s="50"/>
+      <c r="B149" s="52"/>
+      <c r="C149" s="55"/>
       <c r="D149" s="7" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="19"/>
-      <c r="B150" s="49"/>
-      <c r="C150" s="50"/>
+      <c r="B150" s="52"/>
+      <c r="C150" s="55"/>
       <c r="D150" s="7" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="19"/>
-      <c r="B151" s="49"/>
-      <c r="C151" s="50"/>
+      <c r="B151" s="52"/>
+      <c r="C151" s="55"/>
       <c r="D151" s="7" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="19"/>
-      <c r="B152" s="49"/>
-      <c r="C152" s="50"/>
+      <c r="B152" s="52"/>
+      <c r="C152" s="55"/>
       <c r="D152" s="7" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="19"/>
-      <c r="B153" s="49"/>
-      <c r="C153" s="50"/>
+      <c r="B153" s="52"/>
+      <c r="C153" s="55"/>
       <c r="D153" s="7" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="19"/>
-      <c r="B154" s="49"/>
-      <c r="C154" s="50"/>
+      <c r="B154" s="52"/>
+      <c r="C154" s="55"/>
       <c r="D154" s="7" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="19"/>
-      <c r="B155" s="49"/>
-      <c r="C155" s="50"/>
+      <c r="B155" s="52"/>
+      <c r="C155" s="55"/>
       <c r="D155" s="7" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="19"/>
-      <c r="B156" s="49"/>
-      <c r="C156" s="50"/>
+      <c r="B156" s="52"/>
+      <c r="C156" s="55"/>
       <c r="D156" s="7" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="20"/>
-      <c r="B157" s="49">
+      <c r="B157" s="52">
         <v>4</v>
       </c>
-      <c r="C157" s="49">
+      <c r="C157" s="52">
         <v>4.0999999999999996</v>
       </c>
       <c r="D157" s="7" t="s">
@@ -6126,32 +6126,32 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="19"/>
-      <c r="B158" s="49"/>
-      <c r="C158" s="49"/>
+      <c r="B158" s="52"/>
+      <c r="C158" s="52"/>
       <c r="D158" s="7" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="19"/>
-      <c r="B159" s="49"/>
-      <c r="C159" s="49"/>
+      <c r="B159" s="52"/>
+      <c r="C159" s="52"/>
       <c r="D159" s="7" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="19"/>
-      <c r="B160" s="49"/>
-      <c r="C160" s="49"/>
+      <c r="B160" s="52"/>
+      <c r="C160" s="52"/>
       <c r="D160" s="7" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="19"/>
-      <c r="B161" s="49"/>
-      <c r="C161" s="49">
+      <c r="B161" s="52"/>
+      <c r="C161" s="52">
         <v>4.2</v>
       </c>
       <c r="D161" s="7" t="s">
@@ -6160,56 +6160,56 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="19"/>
-      <c r="B162" s="49"/>
-      <c r="C162" s="49"/>
+      <c r="B162" s="52"/>
+      <c r="C162" s="52"/>
       <c r="D162" s="7" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="19"/>
-      <c r="B163" s="49"/>
-      <c r="C163" s="49"/>
+      <c r="B163" s="52"/>
+      <c r="C163" s="52"/>
       <c r="D163" s="7" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="19"/>
-      <c r="B164" s="49"/>
-      <c r="C164" s="49"/>
+      <c r="B164" s="52"/>
+      <c r="C164" s="52"/>
       <c r="D164" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="19"/>
-      <c r="B165" s="49"/>
-      <c r="C165" s="49"/>
+      <c r="B165" s="52"/>
+      <c r="C165" s="52"/>
       <c r="D165" s="7" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="19"/>
-      <c r="B166" s="49"/>
-      <c r="C166" s="49"/>
+      <c r="B166" s="52"/>
+      <c r="C166" s="52"/>
       <c r="D166" s="7" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="19"/>
-      <c r="B167" s="49"/>
-      <c r="C167" s="49"/>
+      <c r="B167" s="52"/>
+      <c r="C167" s="52"/>
       <c r="D167" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="19"/>
-      <c r="B168" s="49"/>
-      <c r="C168" s="49">
+      <c r="B168" s="52"/>
+      <c r="C168" s="52">
         <v>4.3</v>
       </c>
       <c r="D168" s="7" t="s">
@@ -6218,48 +6218,48 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="19"/>
-      <c r="B169" s="49"/>
-      <c r="C169" s="49"/>
+      <c r="B169" s="52"/>
+      <c r="C169" s="52"/>
       <c r="D169" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="19"/>
-      <c r="B170" s="49"/>
-      <c r="C170" s="49"/>
+      <c r="B170" s="52"/>
+      <c r="C170" s="52"/>
       <c r="D170" s="7" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="19"/>
-      <c r="B171" s="49"/>
-      <c r="C171" s="49"/>
+      <c r="B171" s="52"/>
+      <c r="C171" s="52"/>
       <c r="D171" s="7" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="19"/>
-      <c r="B172" s="49"/>
-      <c r="C172" s="49"/>
+      <c r="B172" s="52"/>
+      <c r="C172" s="52"/>
       <c r="D172" s="7" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="19"/>
-      <c r="B173" s="49"/>
-      <c r="C173" s="49"/>
+      <c r="B173" s="52"/>
+      <c r="C173" s="52"/>
       <c r="D173" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="19"/>
-      <c r="B174" s="49"/>
-      <c r="C174" s="49">
+      <c r="B174" s="52"/>
+      <c r="C174" s="52">
         <v>4.4000000000000004</v>
       </c>
       <c r="D174" s="7" t="s">
@@ -6268,56 +6268,56 @@
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="19"/>
-      <c r="B175" s="49"/>
-      <c r="C175" s="49"/>
+      <c r="B175" s="52"/>
+      <c r="C175" s="52"/>
       <c r="D175" s="7" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="19"/>
-      <c r="B176" s="49"/>
-      <c r="C176" s="49"/>
+      <c r="B176" s="52"/>
+      <c r="C176" s="52"/>
       <c r="D176" s="7" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" s="19"/>
-      <c r="B177" s="49"/>
-      <c r="C177" s="49"/>
+      <c r="B177" s="52"/>
+      <c r="C177" s="52"/>
       <c r="D177" s="7" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" s="19"/>
-      <c r="B178" s="49"/>
-      <c r="C178" s="49"/>
+      <c r="B178" s="52"/>
+      <c r="C178" s="52"/>
       <c r="D178" s="7" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="19"/>
-      <c r="B179" s="49"/>
-      <c r="C179" s="49"/>
+      <c r="B179" s="52"/>
+      <c r="C179" s="52"/>
       <c r="D179" s="7" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="180" spans="1:4">
       <c r="A180" s="19"/>
-      <c r="B180" s="49"/>
-      <c r="C180" s="49"/>
+      <c r="B180" s="52"/>
+      <c r="C180" s="52"/>
       <c r="D180" s="7" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="181" spans="1:4">
       <c r="A181" s="19"/>
-      <c r="B181" s="49"/>
-      <c r="C181" s="49"/>
+      <c r="B181" s="52"/>
+      <c r="C181" s="52"/>
       <c r="D181" s="7" t="s">
         <v>57</v>
       </c>
@@ -6325,41 +6325,6 @@
   </sheetData>
   <autoFilter ref="A2:J181" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="51">
-    <mergeCell ref="F50:F58"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="F31:F37"/>
-    <mergeCell ref="F38:F45"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E50:E58"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="A3:A58"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="B26:B58"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E37"/>
-    <mergeCell ref="C18:C25"/>
-    <mergeCell ref="G31:G37"/>
-    <mergeCell ref="E38:E45"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="E18:E25"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="F18:F25"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="E3:E11"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="F3:F11"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="C3:C11"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C15:C17"/>
-    <mergeCell ref="C110:C115"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C31:C37"/>
-    <mergeCell ref="C38:C45"/>
-    <mergeCell ref="C50:C58"/>
     <mergeCell ref="C168:C173"/>
     <mergeCell ref="C174:C181"/>
     <mergeCell ref="B3:B25"/>
@@ -6376,6 +6341,41 @@
     <mergeCell ref="C77:C87"/>
     <mergeCell ref="C88:C100"/>
     <mergeCell ref="C101:C109"/>
+    <mergeCell ref="C110:C115"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C31:C37"/>
+    <mergeCell ref="C38:C45"/>
+    <mergeCell ref="C50:C58"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="E3:E11"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="F3:F11"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="C3:C11"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="G31:G37"/>
+    <mergeCell ref="E38:E45"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="E18:E25"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="F18:F25"/>
+    <mergeCell ref="E50:E58"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="A3:A58"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="B26:B58"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E31:E37"/>
+    <mergeCell ref="C18:C25"/>
+    <mergeCell ref="F50:F58"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="F31:F37"/>
+    <mergeCell ref="F38:F45"/>
+    <mergeCell ref="F46:F49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6395,6 +6395,7 @@
     <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">

</xml_diff>